<commit_message>
updated dataset and the corresponding helper files for reading in the dataset
</commit_message>
<xml_diff>
--- a/RQ2_Prompt_Effectiveness_Modeling/results/qualitative/gate1/gate1_qualitative_patterns.xlsx
+++ b/RQ2_Prompt_Effectiveness_Modeling/results/qualitative/gate1/gate1_qualitative_patterns.xlsx
@@ -1025,7 +1025,7 @@
         <v>2</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>0</v>
@@ -1091,7 +1091,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>0</v>
@@ -1157,7 +1157,7 @@
         <v>1</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>0</v>

</xml_diff>